<commit_message>
Refactor Ribbon handler: delegate mapping and export logic to core services
</commit_message>
<xml_diff>
--- a/ExcelTraining.xlsx
+++ b/ExcelTraining.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\Programming\C# programming\ExcelAddIn1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38332A6C-071B-48C8-B6EA-84798119D3FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39C71A35-FD8A-4F87-8479-A7DA1B8E9AE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-15900" yWindow="3390" windowWidth="14400" windowHeight="8640" xr2:uid="{D2739D47-468D-4C4A-A0B1-304A247770A8}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
   <si>
     <t>Alice</t>
   </si>
@@ -52,6 +52,12 @@
   </si>
   <si>
     <t>City</t>
+  </si>
+  <si>
+    <t>Andrej</t>
+  </si>
+  <si>
+    <t>Olsztyn</t>
   </si>
 </sst>
 </file>
@@ -404,7 +410,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{013AD9A7-4D2D-48BF-A9C3-27EAFEC86B02}">
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
@@ -451,6 +457,17 @@
         <v>5</v>
       </c>
     </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5">
+        <v>40</v>
+      </c>
+      <c r="C5" t="s">
+        <v>10</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: implement dynamic XBRL export with Reflection and validation
- Integrated XbrlExportService into the Core layer.
- Implemented Reflection-based XML attribute generation for the Person model.
- Fixed an issue where Nullable types (int?) were ignored during export.
- Added conditional rendering for ValidationErrors (only exported if not empty).
- Cleaned up the project by removing the legacy OnClick.cs file.
- Refactored Ribbon event handling to use a centralized switch-case dispatcher.
- Improved XML output formatting with proper indentation and line breaks.
</commit_message>
<xml_diff>
--- a/ExcelTraining.xlsx
+++ b/ExcelTraining.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\Programming\C# programming\ExcelAddIn1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39C71A35-FD8A-4F87-8479-A7DA1B8E9AE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17200D7A-22F1-4FF7-BC34-AEC3E4B18608}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-15900" yWindow="3390" windowWidth="14400" windowHeight="8640" xr2:uid="{D2739D47-468D-4C4A-A0B1-304A247770A8}"/>
+    <workbookView xWindow="-17610" yWindow="3255" windowWidth="16950" windowHeight="8640" xr2:uid="{D2739D47-468D-4C4A-A0B1-304A247770A8}"/>
   </bookViews>
   <sheets>
     <sheet name="Лист1" sheetId="1" r:id="rId1"/>
@@ -440,7 +440,7 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>25</v>
+        <v>150</v>
       </c>
       <c r="C3" t="s">
         <v>3</v>

</xml_diff>